<commit_message>
docs(cost): React Native mobile, drop Figma, Teams Free (no paid M365)
Dev-tools core $236 -> $150/mo; initial monthly run $1,094. Email via separate provider; Expo EAS optional.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CostEstimate-OneEdu-Board.xlsx
+++ b/docs/CostEstimate-OneEdu-Board.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="150">
   <si>
     <t>One Edu  —  Cloud &amp; Tooling Cost Estimate</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.1</t>
+    <t>2.2</t>
   </si>
   <si>
     <t>Region / OS</t>
@@ -67,13 +67,13 @@
     <t>Initial annual</t>
   </si>
   <si>
-    <t>$1,180</t>
-  </si>
-  <si>
-    <t>$1,745</t>
-  </si>
-  <si>
-    <t>$14,160</t>
+    <t>$1,094</t>
+  </si>
+  <si>
+    <t>$1,659</t>
+  </si>
+  <si>
+    <t>$13,128</t>
   </si>
   <si>
     <t>Cost by category</t>
@@ -118,10 +118,10 @@
     <t>•  Phasing matches the architecture diagram: everything outside the amber “Phase 2” zone is the lean Phase 1 launch.</t>
   </si>
   <si>
-    <t>•  Covers ALL recurring non-manpower cost: Azure + developer tools/SaaS + app-store &amp; developer accounts + domain.</t>
-  </si>
-  <si>
-    <t>•  Azure DevOps (Repos + Boards + Pipelines) is the chosen toolchain — free for the first 5 users — replacing GitHub + Jira.</t>
+    <t>•  Toolchain: Azure DevOps (Repos+Boards+Pipelines, free for 5 users) · React Native (mobile, open-source) · Microsoft Teams Free.</t>
+  </si>
+  <si>
+    <t>•  Email is provided by a separate provider (budget separately); no paid Microsoft 365 in this estimate.</t>
   </si>
   <si>
     <t>•  EXCLUDES: staff salaries / contractor day-rates, and variable payment-gateway fees (~2.9%/transaction).</t>
@@ -322,22 +322,22 @@
     <t>Repos + Boards + Pipelines — first 5 users free</t>
   </si>
   <si>
-    <t>Microsoft 365</t>
-  </si>
-  <si>
-    <t>Business Standard</t>
-  </si>
-  <si>
-    <t>Email, Office, Teams — per user</t>
-  </si>
-  <si>
-    <t>Figma</t>
-  </si>
-  <si>
-    <t>Professional</t>
-  </si>
-  <si>
-    <t>UI/UX design — per editor</t>
+    <t>React Native</t>
+  </si>
+  <si>
+    <t>Open-source</t>
+  </si>
+  <si>
+    <t>Cross-platform mobile (iOS+Android) from one codebase — free</t>
+  </si>
+  <si>
+    <t>Microsoft Teams</t>
+  </si>
+  <si>
+    <t>Free</t>
+  </si>
+  <si>
+    <t>Chat / meetings; email via separate provider (budget separately)</t>
   </si>
   <si>
     <t>1Password</t>
@@ -373,6 +373,15 @@
     <t>Optional (add if needed)</t>
   </si>
   <si>
+    <t>Expo EAS</t>
+  </si>
+  <si>
+    <t>Production</t>
+  </si>
+  <si>
+    <t>Managed mobile builds + OTA updates (free tier also available)</t>
+  </si>
+  <si>
     <t>Extra parallel job</t>
   </si>
   <si>
@@ -388,15 +397,6 @@
     <t>Error monitoring (App Insights covers basics)</t>
   </si>
   <si>
-    <t>Slack</t>
-  </si>
-  <si>
-    <t>Pro</t>
-  </si>
-  <si>
-    <t>Team chat (free tier also viable) — per user</t>
-  </si>
-  <si>
     <t>BrowserStack</t>
   </si>
   <si>
@@ -433,19 +433,22 @@
     <t>•  Phasing matches the architecture diagram: Phase 1 = lean launch; Phase 2 (amber) services added as each module goes live.</t>
   </si>
   <si>
-    <t>•  DEV mirrors UAT on App Service (S1) + Azure SQL (S0) for environment parity; other DEV components stay minimal.</t>
+    <t>•  DEV mirrors UAT on App Service (S1) + Azure SQL (S0) for parity; other DEV components stay minimal.</t>
   </si>
   <si>
     <t>•  PROD HA = 2x App Service (zone-redundant) + Azure SQL built-in in-region HA (no extra cost).</t>
   </si>
   <si>
-    <t>•  Toolchain: Azure DevOps (Repos + Boards + Pipelines) — free for the first 5 users — replaces GitHub + Jira.</t>
+    <t>•  Toolchain: Azure DevOps (Repos+Boards+Pipelines, free for 5 users) replaces GitHub + Jira.</t>
+  </si>
+  <si>
+    <t>•  Mobile built with React Native (one codebase for iOS + Android) — framework is free; optional Expo EAS for managed cloud builds / OTA.</t>
+  </si>
+  <si>
+    <t>•  Collaboration via Microsoft Teams Free; email is handled by a SEPARATE provider and budgeted separately (no paid M365 here). Figma not used.</t>
   </si>
   <si>
     <t>•  Development tools priced for a team of 5 (editable). Claude Team plan included at $100/mo flat as directed.</t>
-  </si>
-  <si>
-    <t>•  Per-seat tools (M365, 1Password, Slack) scale with team size; adjust Qty on the Development Tools sheet.</t>
   </si>
   <si>
     <t>•  App-store &amp; developer accounts: Apple Developer $99/yr (amortised); Google Play $25 one-time.</t>
@@ -1275,13 +1278,13 @@
         <v>29</v>
       </c>
       <c r="C20" s="13">
-        <v>236</v>
+        <v>150</v>
       </c>
       <c r="D20" s="14">
-        <v>186</v>
+        <v>119</v>
       </c>
       <c r="E20" s="13">
-        <v>2832</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.25">
@@ -1289,13 +1292,13 @@
         <v>30</v>
       </c>
       <c r="C21" s="22">
-        <v>1180</v>
+        <v>1094</v>
       </c>
       <c r="D21" s="23">
-        <v>932</v>
+        <v>864</v>
       </c>
       <c r="E21" s="22">
-        <v>14160</v>
+        <v>13128</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.25">
@@ -1303,13 +1306,13 @@
         <v>31</v>
       </c>
       <c r="C22" s="22">
-        <v>1745</v>
+        <v>1659</v>
       </c>
       <c r="D22" s="23">
-        <v>1379</v>
+        <v>1311</v>
       </c>
       <c r="E22" s="22">
-        <v>20940</v>
+        <v>19908</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
@@ -1853,7 +1856,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="36" customWidth="1"/>
+    <col min="7" max="7" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1966,10 +1969,10 @@
         <v>103</v>
       </c>
       <c r="C8" s="29">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="D8" s="28">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E8" s="29">
         <f>C8*D8</f>
@@ -1989,10 +1992,10 @@
         <v>106</v>
       </c>
       <c r="C9" s="29">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D9" s="28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="29">
         <f>C9*D9</f>
@@ -2109,13 +2112,13 @@
     </row>
     <row r="15" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="29">
         <v>99</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="C15" s="29">
-        <v>40</v>
       </c>
       <c r="D15" s="28">
         <v>1</v>
@@ -2127,18 +2130,18 @@
         <f>E15*12</f>
       </c>
       <c r="G15" s="28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="28" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="B16" s="28" t="s">
         <v>122</v>
       </c>
       <c r="C16" s="29">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="D16" s="28">
         <v>1</v>
@@ -2161,10 +2164,10 @@
         <v>125</v>
       </c>
       <c r="C17" s="29">
-        <v>7.25</v>
+        <v>26</v>
       </c>
       <c r="D17" s="28">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E17" s="29">
         <f>C17*D17</f>
@@ -2270,7 +2273,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="108" customWidth="1"/>
@@ -2346,6 +2349,11 @@
         <v>148</v>
       </c>
     </row>
+    <row r="16" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="27" t="s">
+        <v>149</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
docs(cost): highlight app-store publishing licences (Apple $99/yr, Google Play $25 one-time)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CostEstimate-OneEdu-Board.xlsx
+++ b/docs/CostEstimate-OneEdu-Board.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="153">
   <si>
     <t>One Edu  —  Cloud &amp; Tooling Cost Estimate</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.2</t>
+    <t>2.3</t>
   </si>
   <si>
     <t>Region / OS</t>
@@ -112,16 +112,25 @@
     <t>Fully built  (+ Phase 2 add-ons)</t>
   </si>
   <si>
-    <t>One-time (Google Play Developer account)</t>
+    <t>App-store publishing licences  (iOS + Android)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Apple Developer Program</t>
+  </si>
+  <si>
+    <t>$99 / year  (recurring — included in Dev Tools core)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Google Play Developer</t>
+  </si>
+  <si>
+    <t>$25  one-time</t>
   </si>
   <si>
     <t>•  Phasing matches the architecture diagram: everything outside the amber “Phase 2” zone is the lean Phase 1 launch.</t>
   </si>
   <si>
-    <t>•  Toolchain: Azure DevOps (Repos+Boards+Pipelines, free for 5 users) · React Native (mobile, open-source) · Microsoft Teams Free.</t>
-  </si>
-  <si>
-    <t>•  Email is provided by a separate provider (budget separately); no paid Microsoft 365 in this estimate.</t>
+    <t>•  Toolchain: Azure DevOps (free for 5 users) · React Native mobile (open-source) · Microsoft Teams Free. Email via separate provider (budgeted separately).</t>
   </si>
   <si>
     <t>•  EXCLUDES: staff salaries / contractor day-rates, and variable payment-gateway fees (~2.9%/transaction).</t>
@@ -352,10 +361,10 @@
     <t>Apple Developer</t>
   </si>
   <si>
-    <t>Program</t>
-  </si>
-  <si>
-    <t>iOS publishing ($99/yr amortised)</t>
+    <t>Program (annual)</t>
+  </si>
+  <si>
+    <t>iOS APP-STORE LICENCE — $99 / YEAR (recurring), amortised</t>
   </si>
   <si>
     <t>Domain + DNS</t>
@@ -418,7 +427,7 @@
     <t>One-off</t>
   </si>
   <si>
-    <t>One-time registration</t>
+    <t>Android APP-STORE LICENCE — $25 ONE-TIME</t>
   </si>
   <si>
     <t>Assumptions, Scope &amp; Exclusions</t>
@@ -445,13 +454,13 @@
     <t>•  Mobile built with React Native (one codebase for iOS + Android) — framework is free; optional Expo EAS for managed cloud builds / OTA.</t>
   </si>
   <si>
-    <t>•  Collaboration via Microsoft Teams Free; email is handled by a SEPARATE provider and budgeted separately (no paid M365 here). Figma not used.</t>
+    <t>•  App-store publishing licences: Apple Developer Program = $99 / YEAR (recurring, amortised in Dev Tools); Google Play = $25 ONE-TIME.</t>
+  </si>
+  <si>
+    <t>•  Collaboration via Microsoft Teams Free; email handled by a SEPARATE provider, budgeted separately (no paid M365). Figma not used.</t>
   </si>
   <si>
     <t>•  Development tools priced for a team of 5 (editable). Claude Team plan included at $100/mo flat as directed.</t>
-  </si>
-  <si>
-    <t>•  App-store &amp; developer accounts: Apple Developer $99/yr (amortised); Google Play $25 one-time.</t>
   </si>
   <si>
     <t>•  Cost-down levers: 1-3 yr Azure reservations cut App Service + SQL ~30-40%; stop DEV/UAT off-hours; Azure Dev/Test subscription for non-prod.</t>
@@ -474,7 +483,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -522,8 +531,11 @@
       <b/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
+      <b/>
+      <color rgb="FF1F4E79"/>
+    </font>
+    <font>
+      <color rgb="FF1F4E79"/>
     </font>
     <font>
       <i/>
@@ -549,7 +561,7 @@
       <color rgb="FF1F7A3D"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -584,6 +596,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -634,7 +656,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -693,11 +715,15 @@
     <xf numFmtId="165" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -715,18 +741,27 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -735,14 +770,19 @@
     <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1087,7 +1127,7 @@
   <sheetPr>
     <tabColor rgb="FF1F3A5F"/>
   </sheetPr>
-  <dimension ref="B1:E28"/>
+  <dimension ref="B1:E30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1315,48 +1355,60 @@
         <v>19908</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23" s="24" t="s">
+    <row r="24" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="13">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C25" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-    </row>
-    <row r="27" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="25"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
+      <c r="C26" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
     </row>
     <row r="28" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
+      <c r="B28" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="15">
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="C4:E4"/>
@@ -1366,10 +1418,12 @@
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
     <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1389,238 +1443,238 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="A1" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C3" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="31">
+        <v>73</v>
+      </c>
+      <c r="C4" s="31">
+        <v>73</v>
+      </c>
+      <c r="D4" s="31">
+        <v>190</v>
+      </c>
+      <c r="E4" s="31">
+        <v>380</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="33">
+        <v>15</v>
+      </c>
+      <c r="C5" s="33">
+        <v>15</v>
+      </c>
+      <c r="D5" s="33">
+        <v>80</v>
+      </c>
+      <c r="E5" s="33">
+        <v>80</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="31">
+        <v>3</v>
+      </c>
+      <c r="C6" s="31">
+        <v>8</v>
+      </c>
+      <c r="D6" s="31">
+        <v>12</v>
+      </c>
+      <c r="E6" s="31">
+        <v>12</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="33">
+        <v>0</v>
+      </c>
+      <c r="C7" s="33">
+        <v>45</v>
+      </c>
+      <c r="D7" s="33">
+        <v>45</v>
+      </c>
+      <c r="E7" s="33">
+        <v>45</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="31">
+        <v>5</v>
+      </c>
+      <c r="C8" s="31">
+        <v>10</v>
+      </c>
+      <c r="D8" s="31">
+        <v>60</v>
+      </c>
+      <c r="E8" s="31">
+        <v>60</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="33">
+        <v>2</v>
+      </c>
+      <c r="C9" s="33">
+        <v>3</v>
+      </c>
+      <c r="D9" s="33">
+        <v>5</v>
+      </c>
+      <c r="E9" s="33">
+        <v>5</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="31">
+        <v>5</v>
+      </c>
+      <c r="C10" s="31">
+        <v>15</v>
+      </c>
+      <c r="D10" s="31">
         <v>40</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" s="29">
-        <v>73</v>
-      </c>
-      <c r="C4" s="29">
-        <v>73</v>
-      </c>
-      <c r="D4" s="29">
-        <v>190</v>
-      </c>
-      <c r="E4" s="29">
-        <v>380</v>
-      </c>
-      <c r="F4" s="28" t="s">
+      <c r="E10" s="31">
+        <v>40</v>
+      </c>
+      <c r="F10" s="30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="33">
+        <v>0</v>
+      </c>
+      <c r="C11" s="33">
+        <v>0</v>
+      </c>
+      <c r="D11" s="33">
+        <v>35</v>
+      </c>
+      <c r="E11" s="33">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="31">
-        <v>15</v>
-      </c>
-      <c r="C5" s="31">
-        <v>15</v>
-      </c>
-      <c r="D5" s="31">
-        <v>80</v>
-      </c>
-      <c r="E5" s="31">
-        <v>80</v>
-      </c>
-      <c r="F5" s="30" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="29">
-        <v>3</v>
-      </c>
-      <c r="C6" s="29">
-        <v>8</v>
-      </c>
-      <c r="D6" s="29">
-        <v>12</v>
-      </c>
-      <c r="E6" s="29">
-        <v>12</v>
-      </c>
-      <c r="F6" s="28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" s="31">
+      <c r="F11" s="32" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="31">
         <v>0</v>
       </c>
-      <c r="C7" s="31">
-        <v>45</v>
-      </c>
-      <c r="D7" s="31">
-        <v>45</v>
-      </c>
-      <c r="E7" s="31">
-        <v>45</v>
-      </c>
-      <c r="F7" s="30" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="29">
+      <c r="C12" s="31">
+        <v>0</v>
+      </c>
+      <c r="D12" s="31">
+        <v>0</v>
+      </c>
+      <c r="E12" s="31">
+        <v>0</v>
+      </c>
+      <c r="F12" s="30" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="33">
+        <v>0</v>
+      </c>
+      <c r="C13" s="33">
+        <v>0</v>
+      </c>
+      <c r="D13" s="33">
         <v>5</v>
       </c>
-      <c r="C8" s="29">
-        <v>10</v>
-      </c>
-      <c r="D8" s="29">
-        <v>60</v>
-      </c>
-      <c r="E8" s="29">
-        <v>60</v>
-      </c>
-      <c r="F8" s="28" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="31">
-        <v>2</v>
-      </c>
-      <c r="C9" s="31">
-        <v>3</v>
-      </c>
-      <c r="D9" s="31">
+      <c r="E13" s="33">
         <v>5</v>
       </c>
-      <c r="E9" s="31">
-        <v>5</v>
-      </c>
-      <c r="F9" s="30" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="29">
-        <v>5</v>
-      </c>
-      <c r="C10" s="29">
-        <v>15</v>
-      </c>
-      <c r="D10" s="29">
-        <v>40</v>
-      </c>
-      <c r="E10" s="29">
-        <v>40</v>
-      </c>
-      <c r="F10" s="28" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="B11" s="31">
-        <v>0</v>
-      </c>
-      <c r="C11" s="31">
-        <v>0</v>
-      </c>
-      <c r="D11" s="31">
-        <v>35</v>
-      </c>
-      <c r="E11" s="31">
-        <v>45</v>
-      </c>
-      <c r="F11" s="30" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="B12" s="29">
-        <v>0</v>
-      </c>
-      <c r="C12" s="29">
-        <v>0</v>
-      </c>
-      <c r="D12" s="29">
-        <v>0</v>
-      </c>
-      <c r="E12" s="29">
-        <v>0</v>
-      </c>
-      <c r="F12" s="28" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="31">
-        <v>0</v>
-      </c>
-      <c r="C13" s="31">
-        <v>0</v>
-      </c>
-      <c r="D13" s="31">
-        <v>5</v>
-      </c>
-      <c r="E13" s="31">
-        <v>5</v>
-      </c>
-      <c r="F13" s="30" t="s">
-        <v>63</v>
+      <c r="F13" s="32" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B14" s="22">
         <f>SUM(B4:B13)</f>
@@ -1635,207 +1689,207 @@
         <f>SUM(E4:E13)</f>
       </c>
       <c r="F14" s="21" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="32" t="s">
-        <v>70</v>
-      </c>
-      <c r="B17" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C17" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="34">
+      <c r="A17" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="36">
         <v>50</v>
       </c>
-      <c r="F17" s="32" t="s">
-        <v>71</v>
+      <c r="F17" s="34" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D18" s="33" t="s">
-        <v>67</v>
+      <c r="A18" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="35" t="s">
+        <v>70</v>
       </c>
       <c r="E18" s="19">
         <v>60</v>
       </c>
-      <c r="F18" s="35" t="s">
-        <v>73</v>
+      <c r="F18" s="37" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="B19" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D19" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="E19" s="34">
+      <c r="A19" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="36">
         <v>10</v>
       </c>
-      <c r="F19" s="32" t="s">
-        <v>75</v>
+      <c r="F19" s="34" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D20" s="33" t="s">
-        <v>67</v>
+      <c r="A20" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="35" t="s">
+        <v>70</v>
       </c>
       <c r="E20" s="19">
         <v>10</v>
       </c>
-      <c r="F20" s="35" t="s">
-        <v>77</v>
+      <c r="F20" s="37" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
-        <v>78</v>
-      </c>
-      <c r="B21" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D21" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="34">
+      <c r="A21" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" s="36">
         <v>120</v>
       </c>
-      <c r="F21" s="32" t="s">
-        <v>79</v>
+      <c r="F21" s="34" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="35" t="s">
-        <v>80</v>
-      </c>
-      <c r="B22" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="33" t="s">
-        <v>67</v>
+      <c r="A22" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="35" t="s">
+        <v>70</v>
       </c>
       <c r="E22" s="19">
         <v>80</v>
       </c>
-      <c r="F22" s="35" t="s">
-        <v>81</v>
+      <c r="F22" s="37" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="B23" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C23" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D23" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="E23" s="34">
+      <c r="A23" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="E23" s="36">
         <v>160</v>
       </c>
-      <c r="F23" s="32" t="s">
-        <v>83</v>
+      <c r="F23" s="34" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="35" t="s">
-        <v>84</v>
-      </c>
-      <c r="B24" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="33" t="s">
-        <v>67</v>
+      <c r="A24" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" s="35" t="s">
+        <v>70</v>
       </c>
       <c r="E24" s="19">
         <v>75</v>
       </c>
-      <c r="F24" s="35" t="s">
-        <v>85</v>
+      <c r="F24" s="37" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E25" s="22">
         <f>SUM(E17:E24)</f>
       </c>
       <c r="F25" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1860,39 +1914,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
+      <c r="A1" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
-        <v>88</v>
+      <c r="A2" s="38" t="s">
+        <v>91</v>
       </c>
       <c r="B2" s="21">
         <v>5</v>
       </c>
-      <c r="C2" s="37" t="s">
-        <v>89</v>
+      <c r="C2" s="39" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>22</v>
@@ -1901,193 +1955,193 @@
         <v>24</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-    </row>
-    <row r="6" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>97</v>
-      </c>
-      <c r="C6" s="41">
+      <c r="A5" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+    </row>
+    <row r="6" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="42" t="s">
         <v>100</v>
       </c>
-      <c r="D6" s="40">
+      <c r="C6" s="43">
+        <v>100</v>
+      </c>
+      <c r="D6" s="42">
         <v>1</v>
       </c>
-      <c r="E6" s="41">
+      <c r="E6" s="43">
         <f>C6*D6</f>
       </c>
-      <c r="F6" s="41">
+      <c r="F6" s="43">
         <f>E6*12</f>
       </c>
-      <c r="G6" s="40" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="29">
+      <c r="G6" s="42" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="31">
         <v>0</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="30">
         <v>5</v>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="31">
         <f>C7*D7</f>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="31">
         <f>E7*12</f>
       </c>
-      <c r="G7" s="28" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="29">
+      <c r="G7" s="30" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="31">
         <v>0</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="30">
         <v>1</v>
       </c>
-      <c r="E8" s="29">
+      <c r="E8" s="31">
         <f>C8*D8</f>
       </c>
-      <c r="F8" s="29">
+      <c r="F8" s="31">
         <f>E8*12</f>
       </c>
-      <c r="G8" s="28" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="28" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="29">
+      <c r="G8" s="30" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="31">
         <v>0</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="30">
         <v>1</v>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="31">
         <f>C9*D9</f>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="31">
         <f>E9*12</f>
       </c>
-      <c r="G9" s="28" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" s="29">
+      <c r="G9" s="30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="31">
         <v>8</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="30">
         <v>5</v>
       </c>
-      <c r="E10" s="29">
+      <c r="E10" s="31">
         <f>C10*D10</f>
       </c>
-      <c r="F10" s="29">
+      <c r="F10" s="31">
         <f>E10*12</f>
       </c>
-      <c r="G10" s="28" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="C11" s="29">
+      <c r="G10" s="30" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="B11" s="45" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" s="46">
         <v>8.25</v>
       </c>
-      <c r="D11" s="28">
+      <c r="D11" s="45">
         <v>1</v>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="46">
         <f>C11*D11</f>
       </c>
-      <c r="F11" s="29">
+      <c r="F11" s="46">
         <f>E11*12</f>
       </c>
-      <c r="G11" s="28" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28" t="s">
-        <v>114</v>
-      </c>
-      <c r="B12" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" s="29">
+      <c r="G11" s="45" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" s="31">
         <v>1.25</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="30">
         <v>1</v>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="31">
         <f>C12*D12</f>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="31">
         <f>E12*12</f>
       </c>
-      <c r="G12" s="28" t="s">
-        <v>116</v>
+      <c r="G12" s="30" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E13" s="22">
         <f>SUM(E6:E12)</f>
@@ -2096,167 +2150,167 @@
         <f>SUM(F6:F12)</f>
       </c>
       <c r="G13" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="42" t="s">
-        <v>118</v>
-      </c>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-    </row>
-    <row r="15" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>120</v>
-      </c>
-      <c r="C15" s="29">
+      <c r="A14" s="47" t="s">
+        <v>121</v>
+      </c>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+    </row>
+    <row r="15" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="31">
         <v>99</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="30">
         <v>1</v>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="31">
         <f>C15*D15</f>
       </c>
-      <c r="F15" s="29">
+      <c r="F15" s="31">
         <f>E15*12</f>
       </c>
-      <c r="G15" s="28" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="B16" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="C16" s="29">
+      <c r="G15" s="30" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" s="31">
         <v>40</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="30">
         <v>1</v>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="31">
         <f>C16*D16</f>
       </c>
-      <c r="F16" s="29">
+      <c r="F16" s="31">
         <f>E16*12</f>
       </c>
-      <c r="G16" s="28" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="28" t="s">
-        <v>124</v>
-      </c>
-      <c r="B17" s="28" t="s">
-        <v>125</v>
-      </c>
-      <c r="C17" s="29">
+      <c r="G16" s="30" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="C17" s="31">
         <v>26</v>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="30">
         <v>1</v>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="31">
         <f>C17*D17</f>
       </c>
-      <c r="F17" s="29">
+      <c r="F17" s="31">
         <f>E17*12</f>
       </c>
-      <c r="G17" s="28" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="28" t="s">
-        <v>127</v>
-      </c>
-      <c r="B18" s="28" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="29">
+      <c r="G17" s="30" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="30" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" s="31">
         <v>39</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="30">
         <v>1</v>
       </c>
-      <c r="E18" s="29">
+      <c r="E18" s="31">
         <f>C18*D18</f>
       </c>
-      <c r="F18" s="29">
+      <c r="F18" s="31">
         <f>E18*12</f>
       </c>
-      <c r="G18" s="28" t="s">
-        <v>129</v>
+      <c r="G18" s="30" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="43" t="s">
-        <v>130</v>
-      </c>
-      <c r="B19" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="D19" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="E19" s="44">
+      <c r="A19" s="48" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="49">
         <f>SUM(E15:E18)</f>
       </c>
-      <c r="F19" s="44">
+      <c r="F19" s="49">
         <f>SUM(F15:F18)</f>
       </c>
-      <c r="G19" s="43" t="s">
-        <v>67</v>
+      <c r="G19" s="48" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="42" t="s">
-        <v>131</v>
-      </c>
-      <c r="B20" s="42"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
+      <c r="A20" s="47" t="s">
+        <v>134</v>
+      </c>
+      <c r="B20" s="47"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="47"/>
+      <c r="G20" s="47"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>132</v>
-      </c>
-      <c r="B21" t="s">
-        <v>133</v>
-      </c>
-      <c r="C21" s="13">
+      <c r="A21" s="50" t="s">
+        <v>135</v>
+      </c>
+      <c r="B21" s="51" t="s">
+        <v>136</v>
+      </c>
+      <c r="C21" s="52">
         <v>25</v>
       </c>
-      <c r="D21" s="45">
+      <c r="D21" s="53">
         <v>1</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="52">
         <f>C21*D21</f>
       </c>
       <c r="F21" t="s">
-        <v>67</v>
-      </c>
-      <c r="G21" t="s">
-        <v>134</v>
+        <v>70</v>
+      </c>
+      <c r="G21" s="51" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -2280,78 +2334,78 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>135</v>
+      <c r="A1" s="28" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
-        <v>136</v>
+      <c r="A3" s="29" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>137</v>
+      <c r="A4" s="29" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
-        <v>138</v>
+      <c r="A5" s="29" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>139</v>
+      <c r="A6" s="29" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>140</v>
+      <c r="A7" s="29" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>141</v>
+      <c r="A8" s="29" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>142</v>
+      <c r="A9" s="29" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
-        <v>143</v>
+      <c r="A10" s="29" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
-        <v>144</v>
+      <c r="A11" s="29" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
-        <v>145</v>
+      <c r="A12" s="29" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
-        <v>146</v>
+      <c r="A13" s="29" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
-        <v>147</v>
+      <c r="A14" s="29" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
-        <v>148</v>
+      <c r="A15" s="29" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="27" t="s">
-        <v>149</v>
+      <c r="A16" s="29" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
enhance modules and convert to Uk names
</commit_message>
<xml_diff>
--- a/docs/CostEstimate-OneEdu-Board.xlsx
+++ b/docs/CostEstimate-OneEdu-Board.xlsx
@@ -31,13 +31,13 @@
     <t>Date</t>
   </si>
   <si>
-    <t>June 2026</t>
+    <t>July 2026</t>
   </si>
   <si>
     <t>Version</t>
   </si>
   <si>
-    <t>2.3</t>
+    <t>2.4</t>
   </si>
   <si>
     <t>Region / OS</t>
@@ -67,13 +67,13 @@
     <t>Initial annual</t>
   </si>
   <si>
-    <t>$1,094</t>
-  </si>
-  <si>
-    <t>$1,659</t>
-  </si>
-  <si>
-    <t>$13,128</t>
+    <t>$1,268</t>
+  </si>
+  <si>
+    <t>$1,876</t>
+  </si>
+  <si>
+    <t>$15,216</t>
   </si>
   <si>
     <t>Cost by category</t>
@@ -436,7 +436,7 @@
     <t>•  Scope: ONE tenant (single institution), ~5,000 students + parents + ~300 staff; ~300-500 peak concurrent users (PROD).</t>
   </si>
   <si>
-    <t>•  Region UK South; OS Windows; pay-as-you-go list prices; 730 hrs/month; USD (GBP indicative @ 0.79).</t>
+    <t>•  Region UK South; OS Windows; pay-as-you-go list prices; 730 hrs/month; USD (GBP indicative @ 0.79). Compute repriced at UK South rates (Jul 2026): App Service S1 $0.125/hr, P1v3 $0.333/hr; SQL S0 $0.605/day, S2 $3.025/day — from the Azure Retail Prices API. UK South runs ~20-25% above East US on App Service/SQL; Front Door is global (unchanged); Phase 2 region-priced items carry a +10% UK uplift.</t>
   </si>
   <si>
     <t>•  Phasing matches the architecture diagram: Phase 1 = lean launch; Phase 2 (amber) services added as each module goes live.</t>
@@ -1262,13 +1262,13 @@
         <v>25</v>
       </c>
       <c r="C16" s="13">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="D16" s="14">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="E16" s="13">
-        <v>1236</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
@@ -1276,13 +1276,13 @@
         <v>26</v>
       </c>
       <c r="C17" s="16">
-        <v>169</v>
+        <v>194</v>
       </c>
       <c r="D17" s="17">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="E17" s="16">
-        <v>2028</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
@@ -1290,13 +1290,13 @@
         <v>27</v>
       </c>
       <c r="C18" s="13">
-        <v>672</v>
+        <v>799</v>
       </c>
       <c r="D18" s="14">
-        <v>531</v>
+        <v>631</v>
       </c>
       <c r="E18" s="13">
-        <v>8064</v>
+        <v>9588</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
@@ -1304,13 +1304,13 @@
         <v>28</v>
       </c>
       <c r="C19" s="19">
-        <v>565</v>
+        <v>608</v>
       </c>
       <c r="D19" s="20">
-        <v>446</v>
+        <v>480</v>
       </c>
       <c r="E19" s="19">
-        <v>6780</v>
+        <v>7296</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
@@ -1332,13 +1332,13 @@
         <v>30</v>
       </c>
       <c r="C21" s="22">
-        <v>1094</v>
+        <v>1268</v>
       </c>
       <c r="D21" s="23">
-        <v>864</v>
+        <v>1002</v>
       </c>
       <c r="E21" s="22">
-        <v>13128</v>
+        <v>15216</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.25">
@@ -1346,13 +1346,13 @@
         <v>31</v>
       </c>
       <c r="C22" s="22">
-        <v>1659</v>
+        <v>1876</v>
       </c>
       <c r="D22" s="23">
-        <v>1311</v>
+        <v>1482</v>
       </c>
       <c r="E22" s="22">
-        <v>19908</v>
+        <v>22512</v>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
@@ -1477,16 +1477,16 @@
         <v>47</v>
       </c>
       <c r="B4" s="31">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="C4" s="31">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="D4" s="31">
-        <v>190</v>
+        <v>243</v>
       </c>
       <c r="E4" s="31">
-        <v>380</v>
+        <v>486</v>
       </c>
       <c r="F4" s="30" t="s">
         <v>48</v>
@@ -1497,16 +1497,16 @@
         <v>49</v>
       </c>
       <c r="B5" s="33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5" s="33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D5" s="33">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="E5" s="33">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="F5" s="32" t="s">
         <v>50</v>
@@ -1520,13 +1520,13 @@
         <v>3</v>
       </c>
       <c r="C6" s="31">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="31">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" s="31">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" s="30" t="s">
         <v>52</v>
@@ -1597,16 +1597,16 @@
         <v>59</v>
       </c>
       <c r="B10" s="31">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="31">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D10" s="31">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E10" s="31">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F10" s="30" t="s">
         <v>60</v>
@@ -1678,15 +1678,19 @@
       </c>
       <c r="B14" s="22">
         <f>SUM(B4:B13)</f>
+        <v>125</v>
       </c>
       <c r="C14" s="22">
         <f>SUM(C4:C13)</f>
+        <v>194</v>
       </c>
       <c r="D14" s="22">
         <f>SUM(D4:D13)</f>
+        <v>546</v>
       </c>
       <c r="E14" s="22">
         <f>SUM(E4:E13)</f>
+        <v>799</v>
       </c>
       <c r="F14" s="21" t="s">
         <v>68</v>
@@ -1726,7 +1730,7 @@
         <v>70</v>
       </c>
       <c r="E17" s="36">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F17" s="34" t="s">
         <v>74</v>
@@ -1746,7 +1750,7 @@
         <v>70</v>
       </c>
       <c r="E18" s="19">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F18" s="37" t="s">
         <v>76</v>
@@ -1766,7 +1770,7 @@
         <v>70</v>
       </c>
       <c r="E19" s="36">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F19" s="34" t="s">
         <v>78</v>
@@ -1826,7 +1830,7 @@
         <v>70</v>
       </c>
       <c r="E22" s="19">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="F22" s="37" t="s">
         <v>84</v>
@@ -1846,7 +1850,7 @@
         <v>70</v>
       </c>
       <c r="E23" s="36">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="F23" s="34" t="s">
         <v>86</v>
@@ -1866,7 +1870,7 @@
         <v>70</v>
       </c>
       <c r="E24" s="19">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="F24" s="37" t="s">
         <v>88</v>
@@ -1887,6 +1891,7 @@
       </c>
       <c r="E25" s="22">
         <f>SUM(E17:E24)</f>
+        <v>608</v>
       </c>
       <c r="F25" s="21" t="s">
         <v>70</v>

</xml_diff>